<commit_message>
Fix validation issues: sort CSVs, regenerate XLSX wide format, add missing xlsx
- meat-production-by-region: sort EN/MN CSVs by (year, value) so
  positional numeric comparison passes [4.14, 8.7]
- meat-production-by-region: regenerate XLSX in wide format (years as
  columns) [5.5]
- meat-production-historical-by-type: same CSV sort fix [4.14, 8.7]
- meat-production-historical-by-type: regenerate XLSX in wide format [5.5]
- meat-production-total: create missing meat-production-total.xlsx [1.5]

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/meat-production-by-region.xlsx
+++ b/data.mn/public/datasets/meat-production-by-region.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,346 +413,318 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
-          <t>year</t>
+          <t>Region</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="F1" t="n">
+        <v>2014</v>
+      </c>
+      <c r="G1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H1" t="n">
+        <v>2016</v>
+      </c>
+      <c r="I1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="L1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="M1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="N1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="O1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="P1" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Central region</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B2" t="n">
+        <v>74919.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>66195.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>68650</v>
+      </c>
+      <c r="E2" t="n">
+        <v>76901.89999999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>74263.60000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>118371.9</v>
+      </c>
+      <c r="H2" t="n">
+        <v>108614.3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>107362.9</v>
+      </c>
+      <c r="J2" t="n">
+        <v>121236.9</v>
+      </c>
+      <c r="K2" t="n">
+        <v>125109.2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>156941.4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>141665.8</v>
+      </c>
+      <c r="N2" t="n">
+        <v>164404.8</v>
+      </c>
+      <c r="O2" t="n">
+        <v>173757.3</v>
+      </c>
+      <c r="P2" t="n">
+        <v>121646.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Eastern region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B3" t="n">
+        <v>30486</v>
+      </c>
+      <c r="C3" t="n">
+        <v>48816.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>48601.6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>48400.8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>47545.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>64695.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>71545.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>43860.2</v>
+      </c>
+      <c r="J3" t="n">
+        <v>82776.39999999999</v>
+      </c>
+      <c r="K3" t="n">
+        <v>95406.10000000001</v>
+      </c>
+      <c r="L3" t="n">
+        <v>106995.4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>84610.10000000001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>106085.5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>115241.4</v>
+      </c>
+      <c r="P3" t="n">
+        <v>58589</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Khangai region</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="B4" t="n">
+        <v>82585.7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>90042.89999999999</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95589.10000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>111459.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>107655.9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>168339.1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>137929.3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>175058.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>184093.6</v>
+      </c>
+      <c r="K4" t="n">
+        <v>203005.9</v>
+      </c>
+      <c r="L4" t="n">
+        <v>313579.5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>174359.3</v>
+      </c>
+      <c r="N4" t="n">
+        <v>205303.2</v>
+      </c>
+      <c r="O4" t="n">
+        <v>216948.7</v>
+      </c>
+      <c r="P4" t="n">
+        <v>176453.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Ulaanbaatar</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="B5" t="n">
+        <v>5960.3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5652.8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5198.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5692.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4854.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8709.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>7647.1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8626.4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>9532.700000000001</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8094.4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>7410.6</v>
+      </c>
+      <c r="M5" t="n">
+        <v>9341.299999999999</v>
+      </c>
+      <c r="N5" t="n">
+        <v>9161.299999999999</v>
+      </c>
+      <c r="O5" t="n">
+        <v>6492.6</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5149.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Western region</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B2" t="n">
-        <v>74919.5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30486</v>
-      </c>
-      <c r="D2" t="n">
-        <v>82585.7</v>
-      </c>
-      <c r="E2" t="n">
-        <v>5960.3</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="B6" t="n">
         <v>47118.5</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B3" t="n">
-        <v>66195.5</v>
-      </c>
-      <c r="C3" t="n">
-        <v>48816.7</v>
-      </c>
-      <c r="D3" t="n">
-        <v>90042.89999999999</v>
-      </c>
-      <c r="E3" t="n">
-        <v>5652.8</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="C6" t="n">
         <v>40640</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B4" t="n">
-        <v>68650</v>
-      </c>
-      <c r="C4" t="n">
-        <v>48601.6</v>
-      </c>
-      <c r="D4" t="n">
-        <v>95589.10000000001</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5198.9</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="D6" t="n">
         <v>45375.9</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B5" t="n">
-        <v>76901.89999999999</v>
-      </c>
-      <c r="C5" t="n">
-        <v>48400.8</v>
-      </c>
-      <c r="D5" t="n">
-        <v>111459.4</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5692.3</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="E6" t="n">
         <v>56826.4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B6" t="n">
-        <v>74263.60000000001</v>
-      </c>
-      <c r="C6" t="n">
-        <v>47545.1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>107655.9</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4854.5</v>
       </c>
       <c r="F6" t="n">
         <v>57336.7</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B7" t="n">
-        <v>118371.9</v>
-      </c>
-      <c r="C7" t="n">
-        <v>64695.4</v>
-      </c>
-      <c r="D7" t="n">
-        <v>168339.1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8709.6</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="G6" t="n">
         <v>88039.8</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B8" t="n">
-        <v>108614.3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>71545.2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>137929.3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>7647.1</v>
-      </c>
-      <c r="F8" t="n">
+      <c r="H6" t="n">
         <v>75848.7</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B9" t="n">
-        <v>107362.9</v>
-      </c>
-      <c r="C9" t="n">
-        <v>43860.2</v>
-      </c>
-      <c r="D9" t="n">
-        <v>175058.9</v>
-      </c>
-      <c r="E9" t="n">
-        <v>8626.4</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="I6" t="n">
         <v>91259.89999999999</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B10" t="n">
-        <v>121236.9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>82776.39999999999</v>
-      </c>
-      <c r="D10" t="n">
-        <v>184093.6</v>
-      </c>
-      <c r="E10" t="n">
-        <v>9532.700000000001</v>
-      </c>
-      <c r="F10" t="n">
+      <c r="J6" t="n">
         <v>117543.1</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B11" t="n">
-        <v>125109.2</v>
-      </c>
-      <c r="C11" t="n">
-        <v>95406.10000000001</v>
-      </c>
-      <c r="D11" t="n">
-        <v>203005.9</v>
-      </c>
-      <c r="E11" t="n">
-        <v>8094.4</v>
-      </c>
-      <c r="F11" t="n">
+      <c r="K6" t="n">
         <v>113413.6</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B12" t="n">
-        <v>156941.4</v>
-      </c>
-      <c r="C12" t="n">
-        <v>106995.4</v>
-      </c>
-      <c r="D12" t="n">
-        <v>313579.5</v>
-      </c>
-      <c r="E12" t="n">
-        <v>7410.6</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="L6" t="n">
         <v>159589.1</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B13" t="n">
-        <v>141665.8</v>
-      </c>
-      <c r="C13" t="n">
-        <v>84610.10000000001</v>
-      </c>
-      <c r="D13" t="n">
-        <v>174359.3</v>
-      </c>
-      <c r="E13" t="n">
-        <v>9341.299999999999</v>
-      </c>
-      <c r="F13" t="n">
+      <c r="M6" t="n">
         <v>102702.7</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B14" t="n">
-        <v>164404.8</v>
-      </c>
-      <c r="C14" t="n">
-        <v>106085.5</v>
-      </c>
-      <c r="D14" t="n">
-        <v>205303.2</v>
-      </c>
-      <c r="E14" t="n">
-        <v>9161.299999999999</v>
-      </c>
-      <c r="F14" t="n">
+      <c r="N6" t="n">
         <v>169011.8</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B15" t="n">
-        <v>173757.3</v>
-      </c>
-      <c r="C15" t="n">
-        <v>115241.4</v>
-      </c>
-      <c r="D15" t="n">
-        <v>216948.7</v>
-      </c>
-      <c r="E15" t="n">
-        <v>6492.6</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="O6" t="n">
         <v>109642.8</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B16" t="n">
-        <v>121646.6</v>
-      </c>
-      <c r="C16" t="n">
-        <v>58589</v>
-      </c>
-      <c r="D16" t="n">
-        <v>176453.7</v>
-      </c>
-      <c r="E16" t="n">
-        <v>5149.7</v>
-      </c>
-      <c r="F16" t="n">
+      <c r="P6" t="n">
         <v>88604.10000000001</v>
       </c>
     </row>

</xml_diff>